<commit_message>
Initial commit - Laravel project
</commit_message>
<xml_diff>
--- a/public/templates/template_data_siswa.xlsx
+++ b/public/templates/template_data_siswa.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="sip, lanjut" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="sip, lanjut" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,9 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>nis</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+  <si>
+    <t>nisn</t>
+  </si>
+  <si>
+    <t>nik</t>
   </si>
   <si>
     <t>nama_lengkap</t>
@@ -22,9 +25,6 @@
     <t>jenis_kelamin</t>
   </si>
   <si>
-    <t>nisn</t>
-  </si>
-  <si>
     <t>tempat_lahir</t>
   </si>
   <si>
@@ -38,13 +38,85 @@
   </si>
   <si>
     <t>alamat</t>
+  </si>
+  <si>
+    <t>rombel</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>3201123456780001</t>
+  </si>
+  <si>
+    <t>Budi Santoso</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Jakarta</t>
+  </si>
+  <si>
+    <t>Pak Santoso</t>
+  </si>
+  <si>
+    <t>Jl. Merdeka No. 1</t>
+  </si>
+  <si>
+    <t>1A</t>
+  </si>
+  <si>
+    <t>budi@gmail.com</t>
+  </si>
+  <si>
+    <t>3201123456780002</t>
+  </si>
+  <si>
+    <t>Siti Aminah</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Bandung</t>
+  </si>
+  <si>
+    <t>Ibu Aminah</t>
+  </si>
+  <si>
+    <t>Jl. Mawar No. 10</t>
+  </si>
+  <si>
+    <t>3201123456780003</t>
+  </si>
+  <si>
+    <t>Rizky Ramadhan</t>
+  </si>
+  <si>
+    <t>Surabaya</t>
+  </si>
+  <si>
+    <t>Pak Rizky</t>
+  </si>
+  <si>
+    <t>Jl. Melati No. 5</t>
+  </si>
+  <si>
+    <t>2B</t>
+  </si>
+  <si>
+    <t>rizky.r@yahoo.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -52,8 +124,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <b/>
+      <color rgb="FF1F1F1F"/>
+      <name val="&quot;Google Sans Text&quot;"/>
+    </font>
+    <font>
+      <color rgb="FF1F1F1F"/>
+      <name val="&quot;Google Sans Text&quot;"/>
     </font>
   </fonts>
   <fills count="2">
@@ -70,14 +147,20 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -88,6 +171,10 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -322,17 +409,116 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="G2" s="1"/>
+      <c r="A2" s="2">
+        <v>1.23456789E9</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3">
+        <v>42144.0</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2">
+        <v>8.123456789E9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2">
+        <v>9.87654321E8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3">
+        <v>42233.0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="2">
+        <v>8.129876543E9</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="4"/>
     </row>
-    <row r="4" ht="15.75" customHeight="1"/>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="2">
+        <v>1.122334455E9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="3">
+        <v>41974.0</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="2">
+        <v>8.1311223344E10</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
     <row r="5" ht="15.75" customHeight="1"/>
     <row r="6" ht="15.75" customHeight="1"/>
     <row r="7" ht="15.75" customHeight="1"/>

</xml_diff>